<commit_message>
Added forest mode parameter to control table
</commit_message>
<xml_diff>
--- a/SweForFacilytyData2601.xlsx
+++ b/SweForFacilytyData2601.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\ljeraa\BioFrame\SweForGit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED95A51-7A53-4242-A7F0-367D9E7E9E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868A1CA2-1B91-4DEA-A582-1799C5AA7A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1275" yWindow="780" windowWidth="20490" windowHeight="10950" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19860" windowHeight="12225" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="9" r:id="rId1"/>
@@ -24520,7 +24520,7 @@
         <v>CHPpl_</v>
       </c>
       <c r="L323" s="14">
-        <f t="shared" ref="L323:L386" si="361">IF(K323="-","-",F323*X323)</f>
+        <f t="shared" ref="L323:L359" si="361">IF(K323="-","-",F323*X323)</f>
         <v>0</v>
       </c>
       <c r="V323" s="1">

</xml_diff>